<commit_message>
mobile: Manage chat flag and the moderateChat feature (E9.F1.S14)
authCanManageChat = 0x200, authAllFlags widened to 0x3ff so the app-access
editor no longer strips the new bit, and KennelFeature.moderateChat
(GM | Web Meister, or the flag) in a new PermissionArea.chat. Nothing calls
canEnterArea for 'chat', so the area adds no empty admin doorway: a
moderator acts inside the chat, on the rows the server marks canDelete.
"Manage chat" is added to the app-access editor.

docs/permissions_matrix.xlsx gains a "Delete any chat message" column
(Super Admin, GM, Web Meister) and a Function Reference row, edited in
place because the generator must not be re-run over the hand-filled
workbook; the generator's data is updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGP8euTvGyGJ9z4CT8KTfG
</commit_message>
<xml_diff>
--- a/docs/permissions_matrix.xlsx
+++ b/docs/permissions_matrix.xlsx
@@ -146,7 +146,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -168,11 +168,55 @@
         <color rgb="00B0B0B0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -287,6 +331,11 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -652,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X28"/>
+  <dimension ref="A1:Y28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -679,6 +728,7 @@
     <col width="4.5" customWidth="1" min="22" max="22"/>
     <col width="4.5" customWidth="1" min="23" max="23"/>
     <col width="4.5" customWidth="1" min="24" max="24"/>
+    <col width="4.5" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="46" customHeight="1">
@@ -695,31 +745,45 @@
           <t>Hash Cash</t>
         </is>
       </c>
+      <c r="C2" s="40" t="n"/>
+      <c r="D2" s="40" t="n"/>
+      <c r="E2" s="41" t="n"/>
       <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Runs &amp; Events</t>
         </is>
       </c>
+      <c r="G2" s="40" t="n"/>
+      <c r="H2" s="40" t="n"/>
+      <c r="I2" s="40" t="n"/>
+      <c r="J2" s="41" t="n"/>
       <c r="K2" s="5" t="inlineStr">
         <is>
           <t>Down Downs &amp; Awards</t>
         </is>
       </c>
+      <c r="L2" s="41" t="n"/>
       <c r="M2" s="6" t="inlineStr">
         <is>
           <t>Members</t>
         </is>
       </c>
+      <c r="N2" s="40" t="n"/>
+      <c r="O2" s="40" t="n"/>
+      <c r="P2" s="41" t="n"/>
       <c r="Q2" s="7" t="inlineStr">
         <is>
           <t>Photos</t>
         </is>
       </c>
+      <c r="R2" s="40" t="n"/>
+      <c r="S2" s="41" t="n"/>
       <c r="T2" s="8" t="inlineStr">
         <is>
           <t>Web / Newsletter</t>
         </is>
       </c>
+      <c r="U2" s="41" t="n"/>
       <c r="V2" s="9" t="inlineStr">
         <is>
           <t>Kennel</t>
@@ -735,6 +799,7 @@
           <t>Chat</t>
         </is>
       </c>
+      <c r="Y2" s="41" t="n"/>
     </row>
     <row r="3" ht="150" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
@@ -857,6 +922,11 @@
           <t>Post event chat message</t>
         </is>
       </c>
+      <c r="Y3" s="21" t="inlineStr">
+        <is>
+          <t>Delete any chat message (moderateChat; flag Manage chat 0x200)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="22" t="inlineStr">
@@ -979,6 +1049,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="Y4" s="23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="22" t="inlineStr">
@@ -1101,6 +1176,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="Y5" s="42" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="22" t="inlineStr">
@@ -1147,6 +1223,7 @@
       <c r="V6" s="24" t="inlineStr"/>
       <c r="W6" s="24" t="inlineStr"/>
       <c r="X6" s="24" t="inlineStr"/>
+      <c r="Y6" s="24" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="25" t="inlineStr">
@@ -1181,6 +1258,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="Y7" s="42" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="25" t="inlineStr">
@@ -1299,6 +1377,11 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="Y8" s="23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="25" t="inlineStr">
@@ -1417,6 +1500,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="Y9" s="42" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="25" t="inlineStr">
@@ -1479,6 +1563,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="Y10" s="42" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
@@ -1521,6 +1606,7 @@
       <c r="V11" s="26" t="inlineStr"/>
       <c r="W11" s="26" t="inlineStr"/>
       <c r="X11" s="26" t="inlineStr"/>
+      <c r="Y11" s="42" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="25" t="inlineStr">
@@ -1563,6 +1649,7 @@
       <c r="V12" s="26" t="inlineStr"/>
       <c r="W12" s="26" t="inlineStr"/>
       <c r="X12" s="26" t="inlineStr"/>
+      <c r="Y12" s="42" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="25" t="inlineStr">
@@ -1617,6 +1704,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="Y13" s="42" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="25" t="inlineStr">
@@ -1651,6 +1739,7 @@
         </is>
       </c>
       <c r="X14" s="26" t="inlineStr"/>
+      <c r="Y14" s="42" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="25" t="inlineStr">
@@ -1701,6 +1790,7 @@
       <c r="V15" s="26" t="inlineStr"/>
       <c r="W15" s="26" t="inlineStr"/>
       <c r="X15" s="26" t="inlineStr"/>
+      <c r="Y15" s="42" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="25" t="inlineStr">
@@ -1739,6 +1829,7 @@
       <c r="V16" s="26" t="inlineStr"/>
       <c r="W16" s="26" t="inlineStr"/>
       <c r="X16" s="26" t="inlineStr"/>
+      <c r="Y16" s="42" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="25" t="inlineStr">
@@ -1785,6 +1876,7 @@
       <c r="V17" s="26" t="inlineStr"/>
       <c r="W17" s="26" t="inlineStr"/>
       <c r="X17" s="26" t="inlineStr"/>
+      <c r="Y17" s="42" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="25" t="inlineStr">
@@ -1823,6 +1915,7 @@
       <c r="V18" s="26" t="inlineStr"/>
       <c r="W18" s="26" t="inlineStr"/>
       <c r="X18" s="26" t="inlineStr"/>
+      <c r="Y18" s="42" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="25" t="inlineStr">
@@ -1865,6 +1958,11 @@
       <c r="V19" s="26" t="inlineStr"/>
       <c r="W19" s="26" t="inlineStr"/>
       <c r="X19" s="26" t="inlineStr"/>
+      <c r="Y19" s="23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="25" t="inlineStr">
@@ -1899,6 +1997,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="Y20" s="42" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="25" t="inlineStr">
@@ -1929,6 +2028,7 @@
       <c r="V21" s="26" t="inlineStr"/>
       <c r="W21" s="26" t="inlineStr"/>
       <c r="X21" s="26" t="inlineStr"/>
+      <c r="Y21" s="42" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="25" t="inlineStr">
@@ -1963,6 +2063,7 @@
       <c r="V22" s="26" t="inlineStr"/>
       <c r="W22" s="26" t="inlineStr"/>
       <c r="X22" s="26" t="inlineStr"/>
+      <c r="Y22" s="42" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="25" t="inlineStr">
@@ -1993,6 +2094,7 @@
       <c r="V23" s="26" t="inlineStr"/>
       <c r="W23" s="26" t="inlineStr"/>
       <c r="X23" s="26" t="inlineStr"/>
+      <c r="Y23" s="42" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="25" t="inlineStr">
@@ -2031,6 +2133,7 @@
       <c r="V24" s="26" t="inlineStr"/>
       <c r="W24" s="26" t="inlineStr"/>
       <c r="X24" s="26" t="inlineStr"/>
+      <c r="Y24" s="42" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="25" t="inlineStr">
@@ -2077,6 +2180,7 @@
       <c r="V25" s="26" t="inlineStr"/>
       <c r="W25" s="26" t="inlineStr"/>
       <c r="X25" s="26" t="inlineStr"/>
+      <c r="Y25" s="42" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="25" t="inlineStr">
@@ -2123,6 +2227,7 @@
       <c r="V26" s="26" t="inlineStr"/>
       <c r="W26" s="26" t="inlineStr"/>
       <c r="X26" s="26" t="inlineStr"/>
+      <c r="Y26" s="42" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="25" t="inlineStr">
@@ -2165,6 +2270,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="Y27" s="42" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="25" t="inlineStr">
@@ -2195,16 +2301,17 @@
       <c r="V28" s="26" t="inlineStr"/>
       <c r="W28" s="26" t="inlineStr"/>
       <c r="X28" s="26" t="inlineStr"/>
+      <c r="Y28" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="T2:U2"/>
+    <mergeCell ref="X2:Y2"/>
     <mergeCell ref="K2:L2"/>
-    <mergeCell ref="X2"/>
+    <mergeCell ref="A1:Y1"/>
     <mergeCell ref="V2"/>
     <mergeCell ref="M2:P2"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="A1:X1"/>
     <mergeCell ref="W2"/>
     <mergeCell ref="Q2:S2"/>
     <mergeCell ref="F2:J2"/>
@@ -2224,7 +2331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2947,8 +3054,41 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="39" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="38" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>Delete any chat message (moderateChat)</t>
+        </is>
+      </c>
+      <c r="C25" s="29" t="inlineStr">
+        <is>
+          <t>deleteChatMessage (+ readers' canDelete)</t>
+        </is>
+      </c>
+      <c r="D25" s="30" t="inlineStr">
+        <is>
+          <t>Own message always; else CheckKennelPermission moderateChat (GM|WebMeister or flag Manage chat 0x200); rooms SuperAdmin only</t>
+        </is>
+      </c>
+      <c r="E25" s="29" t="inlineStr">
+        <is>
+          <t>KennelFeature.moderateChat (display only; canDelete comes from the reader)</t>
+        </is>
+      </c>
+      <c r="F25" s="29" t="inlineStr">
+        <is>
+          <t>E9.F1.S13/S14, 2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="39" t="inlineStr">
         <is>
           <t>* 'admin' = SuperAdmin | Admin, but the current mask (0x40000081) also wrongly includes ManagePublicWebContent (0x80) — see audit.</t>
         </is>

</xml_diff>